<commit_message>
refresh: COSMoS package 2026-07-14
</commit_message>
<xml_diff>
--- a/consumer-bases/interim/PR_DSS_Reachability.xlsx
+++ b/consumer-bases/interim/PR_DSS_Reachability.xlsx
@@ -484,7 +484,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-12 21:38</t>
+          <t>Generated: 2026-08-23 19:06</t>
         </is>
       </c>
     </row>
@@ -866,7 +866,7 @@
         <v>0</v>
       </c>
       <c r="D2" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" s="6" t="n">
         <v>0</v>
@@ -880,7 +880,7 @@
       <c r="H2" s="6" t="n"/>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>RADTHERAPHYBREASTCANCER</t>
+          <t>RADIATIONCANCER; RADTHERAPHYBREASTCANCER</t>
         </is>
       </c>
       <c r="J2" s="6" t="inlineStr">
@@ -2367,13 +2367,13 @@
         </is>
       </c>
       <c r="C46" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D46" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F46" s="6" t="n">
         <v>1</v>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="H46" s="6" t="inlineStr">
         <is>
-          <t>CTSCAN; CTSCANCHEST</t>
+          <t>CTSCAN; CTSCANABDOMIN; CTSCANCHEST; CTSCANPELVIS</t>
         </is>
       </c>
       <c r="I46" s="6" t="n"/>
@@ -3156,7 +3156,7 @@
         <v>0</v>
       </c>
       <c r="D69" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E69" s="6" t="n">
         <v>0</v>
@@ -3170,7 +3170,7 @@
       <c r="H69" s="6" t="n"/>
       <c r="I69" s="6" t="inlineStr">
         <is>
-          <t>RADTHERAPHYBREASTCANCER</t>
+          <t>RADIATIONCANCER; RADTHERAPHYBREASTCANCER</t>
         </is>
       </c>
       <c r="J69" s="6" t="inlineStr">
@@ -3568,7 +3568,7 @@
         <v>0</v>
       </c>
       <c r="D81" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E81" s="6" t="n">
         <v>0</v>
@@ -3580,7 +3580,11 @@
         <v>0</v>
       </c>
       <c r="H81" s="6" t="n"/>
-      <c r="I81" s="6" t="n"/>
+      <c r="I81" s="6" t="inlineStr">
+        <is>
+          <t>SURGBRCAPRESP</t>
+        </is>
+      </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
           <t>no_pr_dss</t>
@@ -3874,7 +3878,7 @@
         <v>0</v>
       </c>
       <c r="D90" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E90" s="6" t="n">
         <v>0</v>
@@ -3886,7 +3890,11 @@
         <v>0</v>
       </c>
       <c r="H90" s="6" t="n"/>
-      <c r="I90" s="6" t="n"/>
+      <c r="I90" s="6" t="inlineStr">
+        <is>
+          <t>SURGBRCAPRESP</t>
+        </is>
+      </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
           <t>no_pr_dss</t>
@@ -4589,7 +4597,7 @@
         </is>
       </c>
       <c r="C111" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D111" s="6" t="n">
         <v>0</v>
@@ -4601,13 +4609,17 @@
         <v>0</v>
       </c>
       <c r="G111" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H111" s="6" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="H111" s="6" t="inlineStr">
+        <is>
+          <t>PHOTOGRAPHY</t>
+        </is>
+      </c>
       <c r="I111" s="6" t="n"/>
       <c r="J111" s="6" t="inlineStr">
         <is>
-          <t>no_pr_dss</t>
+          <t>modality_only</t>
         </is>
       </c>
     </row>
@@ -4966,7 +4978,7 @@
         <v>0</v>
       </c>
       <c r="D122" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E122" s="6" t="n">
         <v>0</v>
@@ -4978,7 +4990,11 @@
         <v>0</v>
       </c>
       <c r="H122" s="6" t="n"/>
-      <c r="I122" s="6" t="n"/>
+      <c r="I122" s="6" t="inlineStr">
+        <is>
+          <t>SURGBRCAPRESP</t>
+        </is>
+      </c>
       <c r="J122" s="6" t="inlineStr">
         <is>
           <t>no_pr_dss</t>
@@ -5201,25 +5217,29 @@
         </is>
       </c>
       <c r="C129" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D129" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E129" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F129" s="6" t="n">
         <v>0</v>
       </c>
       <c r="G129" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H129" s="6" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="H129" s="6" t="inlineStr">
+        <is>
+          <t>SCINTIGRAPHY; SCINTIGRAPHYBONE</t>
+        </is>
+      </c>
       <c r="I129" s="6" t="n"/>
       <c r="J129" s="6" t="inlineStr">
         <is>
-          <t>no_pr_dss</t>
+          <t>right_grain_exists</t>
         </is>
       </c>
     </row>
@@ -6055,7 +6075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6409,25 +6429,25 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>C139186</t>
+          <t>C12664</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>ABDOMINAL REGION</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>CTSCAN</t>
-        </is>
-      </c>
+          <t>ABDOMINAL CAVITY</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>CTSCANABDOMIN</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="n"/>
       <c r="H10" s="6" t="n"/>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>modality_only_anatomy_permitted</t>
+          <t>right_grain</t>
         </is>
       </c>
     </row>
@@ -6444,19 +6464,15 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>C25389</t>
+          <t>C139186</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>CHEST</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>CTSCANCHEST</t>
-        </is>
-      </c>
+          <t>ABDOMINAL REGION</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n"/>
       <c r="F11" s="6" t="inlineStr">
         <is>
           <t>CTSCAN</t>
@@ -6466,7 +6482,7 @@
       <c r="H11" s="6" t="n"/>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>right_grain</t>
+          <t>modality_only_anatomy_permitted</t>
         </is>
       </c>
     </row>
@@ -6483,15 +6499,19 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>C12419</t>
+          <t>C25389</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>HEAD</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="n"/>
+          <t>CHEST</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>CTSCANCHEST</t>
+        </is>
+      </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
           <t>CTSCAN</t>
@@ -6501,7 +6521,7 @@
       <c r="H12" s="6" t="n"/>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>modality_only_anatomy_permitted</t>
+          <t>right_grain</t>
         </is>
       </c>
     </row>
@@ -6518,12 +6538,12 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>C12767</t>
+          <t>C12419</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>PELVIS</t>
+          <t>HEAD</t>
         </is>
       </c>
       <c r="E13" s="6" t="n"/>
@@ -6543,35 +6563,39 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>C16135</t>
+          <t>C17204</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>INTENSITY-MODULATED RADIATION THERAPY</t>
+          <t>CT SCAN</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>C12904</t>
+          <t>C12767</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>AXILLARY LYMPH NODE</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="n"/>
+          <t>PELVIS</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>CTSCANPELVIS</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>CTSCAN</t>
+        </is>
+      </c>
       <c r="G14" s="6" t="n"/>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>RADTHERAPHYBREASTCANCER</t>
-        </is>
-      </c>
+      <c r="H14" s="6" t="n"/>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>procedure_in_vlist</t>
+          <t>right_grain</t>
         </is>
       </c>
     </row>
@@ -6588,12 +6612,12 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>C12971</t>
+          <t>C12904</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>BREAST</t>
+          <t>AXILLARY LYMPH NODE</t>
         </is>
       </c>
       <c r="E15" s="6" t="n"/>
@@ -6623,12 +6647,12 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>C12744</t>
+          <t>C12971</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>LUMBAR VERTEBRA</t>
+          <t>BREAST</t>
         </is>
       </c>
       <c r="E16" s="6" t="n"/>
@@ -6658,12 +6682,12 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>C12903</t>
+          <t>C12744</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>SUPRACLAVICULAR LYMPH NODE</t>
+          <t>LUMBAR VERTEBRA</t>
         </is>
       </c>
       <c r="E17" s="6" t="n"/>
@@ -6683,109 +6707,105 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>C16809</t>
+          <t>C16135</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>MRI</t>
+          <t>INTENSITY-MODULATED RADIATION THERAPY</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>C12439</t>
+          <t>C12903</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>BRAIN</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>MRIBRAIN</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>MRI</t>
-        </is>
-      </c>
+          <t>SUPRACLAVICULAR LYMPH NODE</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="n"/>
-      <c r="H18" s="6" t="n"/>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>RADTHERAPHYBREASTCANCER</t>
+        </is>
+      </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>right_grain</t>
+          <t>procedure_in_vlist</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>C16809</t>
+          <t>C15755</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>MRI</t>
+          <t>LUMPECTOMY</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>C69313</t>
+          <t>C12971</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>CERVICAL SPINE</t>
+          <t>BREAST</t>
         </is>
       </c>
       <c r="E19" s="6" t="n"/>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>MRI</t>
-        </is>
-      </c>
+      <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="n"/>
-      <c r="H19" s="6" t="n"/>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>SURGBRCAPRESP</t>
+        </is>
+      </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>modality_only_anatomy_permitted</t>
+          <t>procedure_in_vlist</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>C16809</t>
+          <t>C15278</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>MRI</t>
+          <t>MODIFIED RADICAL MASTECTOMY</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>C12727</t>
+          <t>C12971</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>HEART</t>
+          <t>BREAST</t>
         </is>
       </c>
       <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>MRI</t>
-        </is>
-      </c>
+      <c r="F20" s="6" t="n"/>
       <c r="G20" s="6" t="n"/>
-      <c r="H20" s="6" t="n"/>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>SURGBRCAPRESP</t>
+        </is>
+      </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>modality_only_anatomy_permitted</t>
+          <t>procedure_in_vlist</t>
         </is>
       </c>
     </row>
@@ -6802,15 +6822,19 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>C69314</t>
+          <t>C12439</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>LUMBAR SPINE</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="n"/>
+          <t>BRAIN</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>MRIBRAIN</t>
+        </is>
+      </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
           <t>MRI</t>
@@ -6820,7 +6844,7 @@
       <c r="H21" s="6" t="n"/>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>modality_only_anatomy_permitted</t>
+          <t>right_grain</t>
         </is>
       </c>
     </row>
@@ -6837,12 +6861,12 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>C12464</t>
+          <t>C69313</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>SPINAL CORD</t>
+          <t>CERVICAL SPINE</t>
         </is>
       </c>
       <c r="E22" s="6" t="n"/>
@@ -6872,12 +6896,12 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>C69315</t>
+          <t>C12727</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>THORACIC SPINE</t>
+          <t>HEART</t>
         </is>
       </c>
       <c r="E23" s="6" t="n"/>
@@ -6897,28 +6921,28 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>C38101</t>
+          <t>C16809</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>X-RAY</t>
+          <t>MRI</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>C139186</t>
+          <t>C69314</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>ABDOMINAL REGION</t>
+          <t>LUMBAR SPINE</t>
         </is>
       </c>
       <c r="E24" s="6" t="n"/>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>XRAY</t>
+          <t>MRI</t>
         </is>
       </c>
       <c r="G24" s="6" t="n"/>
@@ -6932,28 +6956,28 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>C38101</t>
+          <t>C16809</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>X-RAY</t>
+          <t>MRI</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>C69313</t>
+          <t>C12464</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>CERVICAL SPINE</t>
+          <t>SPINAL CORD</t>
         </is>
       </c>
       <c r="E25" s="6" t="n"/>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>XRAY</t>
+          <t>MRI</t>
         </is>
       </c>
       <c r="G25" s="6" t="n"/>
@@ -6967,109 +6991,105 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>C38101</t>
+          <t>C16809</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>X-RAY</t>
+          <t>MRI</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>C25389</t>
+          <t>C69315</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>CHEST</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>XRAYCHEST</t>
-        </is>
-      </c>
+          <t>THORACIC SPINE</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="n"/>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>XRAY</t>
+          <t>MRI</t>
         </is>
       </c>
       <c r="G26" s="6" t="n"/>
       <c r="H26" s="6" t="n"/>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>right_grain</t>
+          <t>modality_only_anatomy_permitted</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>C38101</t>
+          <t>C15279</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>X-RAY</t>
+          <t>RADICAL MASTECTOMY</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>C12419</t>
+          <t>C12971</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>HEAD</t>
+          <t>BREAST</t>
         </is>
       </c>
       <c r="E27" s="6" t="n"/>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>XRAY</t>
-        </is>
-      </c>
+      <c r="F27" s="6" t="n"/>
       <c r="G27" s="6" t="n"/>
-      <c r="H27" s="6" t="n"/>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>SURGBRCAPRESP</t>
+        </is>
+      </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>modality_only_anatomy_permitted</t>
+          <t>procedure_in_vlist</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>C38101</t>
+          <t>C62667</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>X-RAY</t>
+          <t>SCINTIGRAPHY</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>C69314</t>
+          <t>C12366</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>LUMBAR SPINE</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="n"/>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>XRAY</t>
-        </is>
-      </c>
+          <t>BONE</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>SCINTIGRAPHYBONE</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="n"/>
       <c r="G28" s="6" t="n"/>
       <c r="H28" s="6" t="n"/>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>modality_only_anatomy_permitted</t>
+          <t>right_grain</t>
         </is>
       </c>
     </row>
@@ -7086,12 +7106,12 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>C69315</t>
+          <t>C139186</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>THORACIC SPINE</t>
+          <t>ABDOMINAL REGION</t>
         </is>
       </c>
       <c r="E29" s="6" t="n"/>
@@ -7103,6 +7123,185 @@
       <c r="G29" s="6" t="n"/>
       <c r="H29" s="6" t="n"/>
       <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>modality_only_anatomy_permitted</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>C38101</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>X-RAY</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>C69313</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>CERVICAL SPINE</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="n"/>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>XRAY</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="n"/>
+      <c r="H30" s="6" t="n"/>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>modality_only_anatomy_permitted</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>C38101</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>X-RAY</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>C25389</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>CHEST</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>XRAYCHEST</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>XRAY</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="n"/>
+      <c r="H31" s="6" t="n"/>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>right_grain</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>C38101</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>X-RAY</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>C12419</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>HEAD</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="n"/>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>XRAY</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="n"/>
+      <c r="H32" s="6" t="n"/>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>modality_only_anatomy_permitted</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>C38101</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>X-RAY</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>C69314</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>LUMBAR SPINE</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="n"/>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>XRAY</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="n"/>
+      <c r="H33" s="6" t="n"/>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>modality_only_anatomy_permitted</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>C38101</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>X-RAY</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>C69315</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>THORACIC SPINE</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="n"/>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>XRAY</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="n"/>
+      <c r="H34" s="6" t="n"/>
+      <c r="I34" s="6" t="inlineStr">
         <is>
           <t>modality_only_anatomy_permitted</t>
         </is>

</xml_diff>